<commit_message>
Update: Bharuch-April-2026 by admin
</commit_message>
<xml_diff>
--- a/Bharuch-April-2026.xlsx
+++ b/Bharuch-April-2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Accounts\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5099B1-345E-4191-B013-05CB456043E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF578B1A-E4D1-4ADD-BF4B-8704306C6ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6F51AC4A-10DE-4167-BC74-9E39238F7D09}"/>
   </bookViews>
@@ -50,9 +50,6 @@
     <t>Profit %</t>
   </si>
   <si>
-    <t>APRIL</t>
-  </si>
-  <si>
     <t>MH02GH6038</t>
   </si>
   <si>
@@ -129,6 +126,9 @@
   </si>
   <si>
     <t>Bharuch</t>
+  </si>
+  <si>
+    <t>April</t>
   </si>
 </sst>
 </file>
@@ -630,79 +630,79 @@
   <sheetData>
     <row r="1" spans="1:26" s="4" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="O1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="P1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="W1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="X1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y1" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="Z1" s="3" t="s">
         <v>2</v>
@@ -713,19 +713,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>29</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>3</v>
       </c>
       <c r="D2" s="12">
         <v>2026</v>
       </c>
       <c r="E2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="13" t="s">
         <v>4</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>5</v>
       </c>
       <c r="G2" s="14">
         <v>45804</v>

</xml_diff>